<commit_message>
Day 01: Completed Assignment 01
Solved Assignment 01 covering basic Excel formulas including SUM, AVERAGE, IF, COUNT, COUNTA, COUNTIF,  and SUMIF as part of my 50 Days Microsoft Excel Practice Challenge.
</commit_message>
<xml_diff>
--- a/Excel-Assignments-solution.xlsx
+++ b/Excel-Assignments-solution.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Analytics\ReClasses\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7B374333-51A8-4EC3-BE36-BEFFD8DAC623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C02F599C-A0F3-4BA7-88A8-72E5D0C9D375}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7F6CA21F-FA47-42DF-92A2-56BFE6F74A15}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>Assigment-1</t>
   </si>
@@ -115,6 +115,36 @@
   </si>
   <si>
     <t xml:space="preserve">Ans: No of Students having "A" are </t>
+  </si>
+  <si>
+    <t xml:space="preserve">         No of Students having "B" are </t>
+  </si>
+  <si>
+    <t>Q.4: Student Ashok and Manoj Total Number and Average</t>
+  </si>
+  <si>
+    <t>Ans: Total Number</t>
+  </si>
+  <si>
+    <t>Avearage</t>
+  </si>
+  <si>
+    <t>Q.5: Count how many students</t>
+  </si>
+  <si>
+    <t>Ans: Total Students</t>
+  </si>
+  <si>
+    <t>Q.6: How many student Hindi &amp; English Subject Number Greater then &gt;20 and &lt;15.</t>
+  </si>
+  <si>
+    <t>Ans: No of Students having Hindi Subject Number Greater then &gt;20 are</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         No of Students having English Subject Number less then &lt;15 are</t>
+  </si>
+  <si>
+    <t>No of Students having Hindi &amp; English Subject Number Greater then &gt;20 and &lt;15 are</t>
   </si>
 </sst>
 </file>
@@ -469,10 +499,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E77540B2-D6E8-420D-BAD3-66513A92FF36}">
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="13.36328125" customWidth="1"/>
+    <col min="6" max="6" width="9.6328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
@@ -880,28 +911,104 @@
         <v>A</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>26</v>
       </c>
       <c r="D20">
-        <f>COUNTIF($J$6:$J$15,$J6="A")</f>
-        <v>0</v>
+        <f>COUNTIF($J$6:$J$15,"A")</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>27</v>
+      </c>
+      <c r="D21">
+        <f>COUNTIF($J$6:$J$15,"B")</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>29</v>
+      </c>
+      <c r="C23">
+        <f>SUMIF(B6:B15,"ASHOK",H6:H15)+SUMIF(B6:B15,"MANOJ",H6:H15)</f>
+        <v>163</v>
+      </c>
+      <c r="E23" t="s">
+        <v>30</v>
+      </c>
+      <c r="F23">
+        <f>AVERAGE(SUMIF(B6:B15,"ASHOK",I6:I15)+SUMIF(B6:B15,"MANOJ",I6:I15))</f>
+        <v>32.6</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>32</v>
+      </c>
+      <c r="C25">
+        <f>COUNTA(B6:B15)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>34</v>
+      </c>
+      <c r="H27">
+        <f>COUNTIF(C6:C15,"&gt;20")</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>35</v>
+      </c>
+      <c r="G28">
+        <f>COUNTIF(D6:D15,"&lt;15")</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>36</v>
+      </c>
+      <c r="I29">
+        <f>COUNTIFS(C6:C15,"&gt;20",D6:D15,"&lt;15")</f>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Day 02: Assignment 2
Assignment 2 has completed. I used Product, If, Counta,Countif,Xlookup in the Assignment.
</commit_message>
<xml_diff>
--- a/Excel-Assignments-solution.xlsx
+++ b/Excel-Assignments-solution.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Analytics\ReClasses\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C02F599C-A0F3-4BA7-88A8-72E5D0C9D375}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62106C38-55EC-4E56-A7FA-B2EEE8DC5D73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{7F6CA21F-FA47-42DF-92A2-56BFE6F74A15}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{7F6CA21F-FA47-42DF-92A2-56BFE6F74A15}"/>
   </bookViews>
   <sheets>
     <sheet name="Assignment-1" sheetId="1" r:id="rId1"/>
+    <sheet name="Assignment-2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
   <si>
     <t>Assigment-1</t>
   </si>
@@ -145,6 +146,93 @@
   </si>
   <si>
     <t>No of Students having Hindi &amp; English Subject Number Greater then &gt;20 and &lt;15 are</t>
+  </si>
+  <si>
+    <t>Assignment - 2</t>
+  </si>
+  <si>
+    <t>Use of Formulas-Product,If,Counta,Countif,Sumif</t>
+  </si>
+  <si>
+    <t>SRNO</t>
+  </si>
+  <si>
+    <t>ITEMS</t>
+  </si>
+  <si>
+    <t>AC</t>
+  </si>
+  <si>
+    <t>FRIDGE</t>
+  </si>
+  <si>
+    <t>COOLER</t>
+  </si>
+  <si>
+    <t>WASHING MACHINE</t>
+  </si>
+  <si>
+    <t>TV</t>
+  </si>
+  <si>
+    <t>FAN</t>
+  </si>
+  <si>
+    <t>COMPUTER</t>
+  </si>
+  <si>
+    <t>KEYBOARD</t>
+  </si>
+  <si>
+    <t>MOUSE</t>
+  </si>
+  <si>
+    <t>PRINTER</t>
+  </si>
+  <si>
+    <t>QTY</t>
+  </si>
+  <si>
+    <t>RATE</t>
+  </si>
+  <si>
+    <t>AMOUNT</t>
+  </si>
+  <si>
+    <t>Q.1: Using of Product Formula for Calculate Amount=Qty*Rate</t>
+  </si>
+  <si>
+    <t>Q.2: How many Items in a List</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ans: </t>
+  </si>
+  <si>
+    <t>Q.3: How many Items qty Greater then &gt;20 and Less then &lt;20</t>
+  </si>
+  <si>
+    <t>Ans: No of items qty greater then &gt;20 are</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         No of items qty less then &lt;20 are</t>
+  </si>
+  <si>
+    <t>Ans: Qty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Rate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Amount</t>
+  </si>
+  <si>
+    <t>Q.4: Calculate item computer Qty,Rate and amount .</t>
+  </si>
+  <si>
+    <t>Q.5: If items Amount is Greater&gt;500000, Then items "Expensive" otherwise "Lets Buy it".</t>
+  </si>
+  <si>
+    <t>GRADE</t>
   </si>
 </sst>
 </file>
@@ -168,10 +256,36 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -180,11 +294,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1018,4 +1134,359 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AF899099-0CE0-43AA-BF38-3A1414E5E90C}">
+  <dimension ref="A1:F27"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="6" max="6" width="11" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" s="2">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" s="2">
+        <v>20</v>
+      </c>
+      <c r="D5" s="2">
+        <v>40000</v>
+      </c>
+      <c r="E5" s="2">
+        <f>D5*C5</f>
+        <v>800000</v>
+      </c>
+      <c r="F5" t="str">
+        <f>IF(E5&gt;500000,"Expensive","Lets Buy it")</f>
+        <v>Expensive</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" s="2">
+        <v>2</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" s="2">
+        <v>30</v>
+      </c>
+      <c r="D6" s="2">
+        <v>20000</v>
+      </c>
+      <c r="E6" s="2">
+        <f t="shared" ref="E6:E14" si="0">D6*C6</f>
+        <v>600000</v>
+      </c>
+      <c r="F6" t="str">
+        <f t="shared" ref="F6:F14" si="1">IF(E6&gt;500000,"Expensive","Lets Buy it")</f>
+        <v>Expensive</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" s="2">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" s="2">
+        <v>15</v>
+      </c>
+      <c r="D7" s="2">
+        <v>10000</v>
+      </c>
+      <c r="E7" s="2">
+        <f t="shared" si="0"/>
+        <v>150000</v>
+      </c>
+      <c r="F7" t="str">
+        <f t="shared" si="1"/>
+        <v>Lets Buy it</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" s="2">
+        <v>4</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" s="2">
+        <v>14</v>
+      </c>
+      <c r="D8" s="2">
+        <v>15000</v>
+      </c>
+      <c r="E8" s="2">
+        <f t="shared" si="0"/>
+        <v>210000</v>
+      </c>
+      <c r="F8" t="str">
+        <f t="shared" si="1"/>
+        <v>Lets Buy it</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" s="2">
+        <v>5</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" s="2">
+        <v>18</v>
+      </c>
+      <c r="D9" s="2">
+        <v>20000</v>
+      </c>
+      <c r="E9" s="2">
+        <f t="shared" si="0"/>
+        <v>360000</v>
+      </c>
+      <c r="F9" t="str">
+        <f t="shared" si="1"/>
+        <v>Lets Buy it</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" s="2">
+        <v>6</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" s="2">
+        <v>17</v>
+      </c>
+      <c r="D10" s="2">
+        <v>2000</v>
+      </c>
+      <c r="E10" s="2">
+        <f t="shared" si="0"/>
+        <v>34000</v>
+      </c>
+      <c r="F10" t="str">
+        <f t="shared" si="1"/>
+        <v>Lets Buy it</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" s="2">
+        <v>7</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C11" s="2">
+        <v>10</v>
+      </c>
+      <c r="D11" s="2">
+        <v>25000</v>
+      </c>
+      <c r="E11" s="2">
+        <f t="shared" si="0"/>
+        <v>250000</v>
+      </c>
+      <c r="F11" t="str">
+        <f t="shared" si="1"/>
+        <v>Lets Buy it</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" s="2">
+        <v>8</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" s="2">
+        <v>5</v>
+      </c>
+      <c r="D12" s="2">
+        <v>250</v>
+      </c>
+      <c r="E12" s="2">
+        <f t="shared" si="0"/>
+        <v>1250</v>
+      </c>
+      <c r="F12" t="str">
+        <f t="shared" si="1"/>
+        <v>Lets Buy it</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A13" s="2">
+        <v>9</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="2">
+        <v>25</v>
+      </c>
+      <c r="D13" s="2">
+        <v>100</v>
+      </c>
+      <c r="E13" s="2">
+        <f t="shared" si="0"/>
+        <v>2500</v>
+      </c>
+      <c r="F13" t="str">
+        <f t="shared" si="1"/>
+        <v>Lets Buy it</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" s="2">
+        <v>10</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C14" s="2">
+        <v>30</v>
+      </c>
+      <c r="D14" s="2">
+        <v>12000</v>
+      </c>
+      <c r="E14" s="2">
+        <f t="shared" si="0"/>
+        <v>360000</v>
+      </c>
+      <c r="F14" t="str">
+        <f t="shared" si="1"/>
+        <v>Lets Buy it</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>56</v>
+      </c>
+      <c r="B18">
+        <f>COUNTA(B5:B14)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>58</v>
+      </c>
+      <c r="D20">
+        <f>COUNTIF(C5:C14,"&gt;20")</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>59</v>
+      </c>
+      <c r="D21">
+        <f>COUNTIF(C5:C14,"&lt;20")</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>60</v>
+      </c>
+      <c r="B24">
+        <f>_xlfn.XLOOKUP(B11,B5:B14,C5:C14,,0,)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>61</v>
+      </c>
+      <c r="B25">
+        <f>_xlfn.XLOOKUP(B11,B5:B14,D5:D14,,0,)</f>
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>62</v>
+      </c>
+      <c r="B26">
+        <f>_xlfn.XLOOKUP(B11,B5:B14,E5:E14,,0,)</f>
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>64</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Day:03 Assignment-03 has completed.
Assignment -03 has completed . Use of Formulas- Sum, Nestedif, Counta, Countif, Sumif, Vlookup
</commit_message>
<xml_diff>
--- a/Excel-Assignments-solution.xlsx
+++ b/Excel-Assignments-solution.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Analytics\ReClasses\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62106C38-55EC-4E56-A7FA-B2EEE8DC5D73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58C1BE45-EAFF-433A-AD10-12C9594FB201}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{7F6CA21F-FA47-42DF-92A2-56BFE6F74A15}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{7F6CA21F-FA47-42DF-92A2-56BFE6F74A15}"/>
   </bookViews>
   <sheets>
     <sheet name="Assignment-1" sheetId="1" r:id="rId1"/>
     <sheet name="Assignment-2" sheetId="2" r:id="rId2"/>
+    <sheet name="Assignment-3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="87">
   <si>
     <t>Assigment-1</t>
   </si>
@@ -233,6 +234,69 @@
   </si>
   <si>
     <t>GRADE</t>
+  </si>
+  <si>
+    <t>Use of Formulas- Sum,NestedIf,Counta,Countif,Sumif,Vlookup</t>
+  </si>
+  <si>
+    <t>SUBJECT</t>
+  </si>
+  <si>
+    <t>HINDI</t>
+  </si>
+  <si>
+    <t>ENGLISH</t>
+  </si>
+  <si>
+    <t>MATH</t>
+  </si>
+  <si>
+    <t>PHYSICS</t>
+  </si>
+  <si>
+    <t>CHEMISTRY</t>
+  </si>
+  <si>
+    <t>HISTORY</t>
+  </si>
+  <si>
+    <t>GEO</t>
+  </si>
+  <si>
+    <t>BIO</t>
+  </si>
+  <si>
+    <t>BOTANY</t>
+  </si>
+  <si>
+    <t>1ST</t>
+  </si>
+  <si>
+    <t>2ND</t>
+  </si>
+  <si>
+    <t>3RD</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t>Q.1: How many subject?</t>
+  </si>
+  <si>
+    <t>Q.2: How many subject 1 paper greater then 20?</t>
+  </si>
+  <si>
+    <t>AVERAGE</t>
+  </si>
+  <si>
+    <t>Q.3: Subject Hindi,Math and English total no.  And Average</t>
+  </si>
+  <si>
+    <t>Q.4: If Avg. Greater than 20 then "A",If Avg. Greater than 15 "B",otherwise "C"</t>
+  </si>
+  <si>
+    <t>Q.5: Subject Physics,Maths and English Total/Average</t>
   </si>
 </sst>
 </file>
@@ -256,7 +320,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -279,28 +343,16 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -623,22 +675,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -1146,259 +1198,259 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="1" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="2">
+      <c r="A5" s="1">
         <v>1</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="1">
         <v>20</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="1">
         <v>40000</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="1">
         <f>D5*C5</f>
         <v>800000</v>
       </c>
-      <c r="F5" t="str">
+      <c r="F5" s="1" t="str">
         <f>IF(E5&gt;500000,"Expensive","Lets Buy it")</f>
         <v>Expensive</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="2">
+      <c r="A6" s="1">
         <v>2</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="1">
         <v>30</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="1">
         <v>20000</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="1">
         <f t="shared" ref="E6:E14" si="0">D6*C6</f>
         <v>600000</v>
       </c>
-      <c r="F6" t="str">
+      <c r="F6" s="1" t="str">
         <f t="shared" ref="F6:F14" si="1">IF(E6&gt;500000,"Expensive","Lets Buy it")</f>
         <v>Expensive</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A7" s="2">
+      <c r="A7" s="1">
         <v>3</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="1">
         <v>15</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="1">
         <v>10000</v>
       </c>
-      <c r="E7" s="2">
+      <c r="E7" s="1">
         <f t="shared" si="0"/>
         <v>150000</v>
       </c>
-      <c r="F7" t="str">
+      <c r="F7" s="1" t="str">
         <f t="shared" si="1"/>
         <v>Lets Buy it</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A8" s="2">
+      <c r="A8" s="1">
         <v>4</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="1">
         <v>14</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
         <v>15000</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="1">
         <f t="shared" si="0"/>
         <v>210000</v>
       </c>
-      <c r="F8" t="str">
+      <c r="F8" s="1" t="str">
         <f t="shared" si="1"/>
         <v>Lets Buy it</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A9" s="2">
+      <c r="A9" s="1">
         <v>5</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="1">
         <v>18</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="1">
         <v>20000</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="1">
         <f t="shared" si="0"/>
         <v>360000</v>
       </c>
-      <c r="F9" t="str">
+      <c r="F9" s="1" t="str">
         <f t="shared" si="1"/>
         <v>Lets Buy it</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A10" s="2">
+      <c r="A10" s="1">
         <v>6</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="1">
         <v>17</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="1">
         <v>2000</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="1">
         <f t="shared" si="0"/>
         <v>34000</v>
       </c>
-      <c r="F10" t="str">
+      <c r="F10" s="1" t="str">
         <f t="shared" si="1"/>
         <v>Lets Buy it</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A11" s="2">
+      <c r="A11" s="1">
         <v>7</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="1">
         <v>10</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="1">
         <v>25000</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="1">
         <f t="shared" si="0"/>
         <v>250000</v>
       </c>
-      <c r="F11" t="str">
+      <c r="F11" s="1" t="str">
         <f t="shared" si="1"/>
         <v>Lets Buy it</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" s="2">
+      <c r="A12" s="1">
         <v>8</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="1">
         <v>5</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>250</v>
       </c>
-      <c r="E12" s="2">
+      <c r="E12" s="1">
         <f t="shared" si="0"/>
         <v>1250</v>
       </c>
-      <c r="F12" t="str">
+      <c r="F12" s="1" t="str">
         <f t="shared" si="1"/>
         <v>Lets Buy it</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13" s="2">
+      <c r="A13" s="1">
         <v>9</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13" s="1">
         <v>25</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>100</v>
       </c>
-      <c r="E13" s="2">
+      <c r="E13" s="1">
         <f t="shared" si="0"/>
         <v>2500</v>
       </c>
-      <c r="F13" t="str">
+      <c r="F13" s="1" t="str">
         <f t="shared" si="1"/>
         <v>Lets Buy it</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A14" s="2">
+      <c r="A14" s="1">
         <v>10</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C14" s="2">
+      <c r="C14" s="1">
         <v>30</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="1">
         <v>12000</v>
       </c>
-      <c r="E14" s="2">
+      <c r="E14" s="1">
         <f t="shared" si="0"/>
         <v>360000</v>
       </c>
-      <c r="F14" t="str">
+      <c r="F14" s="1" t="str">
         <f t="shared" si="1"/>
         <v>Lets Buy it</v>
       </c>
@@ -1489,4 +1541,340 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8412A87F-02AE-4909-A9E6-088BD6F06133}">
+  <dimension ref="A1:G21"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="11.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B4" s="1">
+        <v>20</v>
+      </c>
+      <c r="C4" s="1">
+        <v>15</v>
+      </c>
+      <c r="D4" s="1">
+        <v>20</v>
+      </c>
+      <c r="E4" s="1">
+        <f>SUM(B4:D4)</f>
+        <v>55</v>
+      </c>
+      <c r="F4" s="1">
+        <f>AVERAGE(B4:D4)</f>
+        <v>18.333333333333332</v>
+      </c>
+      <c r="G4" s="1" t="str">
+        <f>IF(F4&gt;20,"A",IF(F4&gt;15,"B","C"))</f>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B5" s="1">
+        <v>30</v>
+      </c>
+      <c r="C5" s="1">
+        <v>12</v>
+      </c>
+      <c r="D5" s="1">
+        <v>15</v>
+      </c>
+      <c r="E5" s="1">
+        <f t="shared" ref="E5:E12" si="0">SUM(B5:D5)</f>
+        <v>57</v>
+      </c>
+      <c r="F5" s="1">
+        <f t="shared" ref="F5:F12" si="1">AVERAGE(B5:D5)</f>
+        <v>19</v>
+      </c>
+      <c r="G5" s="1" t="str">
+        <f t="shared" ref="G5:G12" si="2">IF(F5&gt;20,"A",IF(F5&gt;15,"B","C"))</f>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B6" s="1">
+        <v>15</v>
+      </c>
+      <c r="C6" s="1">
+        <v>14</v>
+      </c>
+      <c r="D6" s="1">
+        <v>14</v>
+      </c>
+      <c r="E6" s="1">
+        <f t="shared" si="0"/>
+        <v>43</v>
+      </c>
+      <c r="F6" s="1">
+        <f t="shared" si="1"/>
+        <v>14.333333333333334</v>
+      </c>
+      <c r="G6" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B7" s="1">
+        <v>12</v>
+      </c>
+      <c r="C7" s="1">
+        <v>17</v>
+      </c>
+      <c r="D7" s="1">
+        <v>17</v>
+      </c>
+      <c r="E7" s="1">
+        <f t="shared" si="0"/>
+        <v>46</v>
+      </c>
+      <c r="F7" s="1">
+        <f t="shared" si="1"/>
+        <v>15.333333333333334</v>
+      </c>
+      <c r="G7" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="B8" s="1">
+        <v>14</v>
+      </c>
+      <c r="C8" s="1">
+        <v>18</v>
+      </c>
+      <c r="D8" s="1">
+        <v>18</v>
+      </c>
+      <c r="E8" s="1">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
+      <c r="F8" s="1">
+        <f t="shared" si="1"/>
+        <v>16.666666666666668</v>
+      </c>
+      <c r="G8" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B9" s="1">
+        <v>16</v>
+      </c>
+      <c r="C9" s="1">
+        <v>25</v>
+      </c>
+      <c r="D9" s="1">
+        <v>20</v>
+      </c>
+      <c r="E9" s="1">
+        <f t="shared" si="0"/>
+        <v>61</v>
+      </c>
+      <c r="F9" s="1">
+        <f t="shared" si="1"/>
+        <v>20.333333333333332</v>
+      </c>
+      <c r="G9" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="B10" s="1">
+        <v>18</v>
+      </c>
+      <c r="C10" s="1">
+        <v>21</v>
+      </c>
+      <c r="D10" s="1">
+        <v>22</v>
+      </c>
+      <c r="E10" s="1">
+        <f t="shared" si="0"/>
+        <v>61</v>
+      </c>
+      <c r="F10" s="1">
+        <f t="shared" si="1"/>
+        <v>20.333333333333332</v>
+      </c>
+      <c r="G10" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B11" s="1">
+        <v>17</v>
+      </c>
+      <c r="C11" s="1">
+        <v>23</v>
+      </c>
+      <c r="D11" s="1">
+        <v>13</v>
+      </c>
+      <c r="E11" s="1">
+        <f t="shared" si="0"/>
+        <v>53</v>
+      </c>
+      <c r="F11" s="1">
+        <f t="shared" si="1"/>
+        <v>17.666666666666668</v>
+      </c>
+      <c r="G11" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" s="1">
+        <v>20</v>
+      </c>
+      <c r="C12" s="1">
+        <v>25</v>
+      </c>
+      <c r="D12" s="1">
+        <v>25</v>
+      </c>
+      <c r="E12" s="1">
+        <f t="shared" si="0"/>
+        <v>70</v>
+      </c>
+      <c r="F12" s="1">
+        <f t="shared" si="1"/>
+        <v>23.333333333333332</v>
+      </c>
+      <c r="G12" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>A</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>56</v>
+      </c>
+      <c r="B15">
+        <f>COUNTA(A4:A12)</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>56</v>
+      </c>
+      <c r="B17">
+        <f>COUNTIF(B4:B12,"&gt;20")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>56</v>
+      </c>
+      <c r="B21">
+        <f>SUM(E5:E7)/AVERAGE(F5:F7)</f>
+        <v>8.9999999999999982</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Day-04: Assignment-04 has completed.
Assignment-04 has completed. To complete assignment-04, i use of Formulas-Sum, NestedIf, Counta, Countif, Sumif, Vlookup.
</commit_message>
<xml_diff>
--- a/Excel-Assignments-solution.xlsx
+++ b/Excel-Assignments-solution.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Analytics\ReClasses\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58C1BE45-EAFF-433A-AD10-12C9594FB201}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8F9ADB3-8552-4C42-A158-5F08B5A6793C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{7F6CA21F-FA47-42DF-92A2-56BFE6F74A15}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{7F6CA21F-FA47-42DF-92A2-56BFE6F74A15}"/>
   </bookViews>
   <sheets>
     <sheet name="Assignment-1" sheetId="1" r:id="rId1"/>
     <sheet name="Assignment-2" sheetId="2" r:id="rId2"/>
     <sheet name="Assignment-3" sheetId="3" r:id="rId3"/>
+    <sheet name="Assignment-4" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="122">
   <si>
     <t>Assigment-1</t>
   </si>
@@ -297,6 +298,111 @@
   </si>
   <si>
     <t>Q.5: Subject Physics,Maths and English Total/Average</t>
+  </si>
+  <si>
+    <t>Use of Formulas - Sum, NestedIf, Counta, Countif, Sumif, Vlookup</t>
+  </si>
+  <si>
+    <t>NAME</t>
+  </si>
+  <si>
+    <t>SHYAM</t>
+  </si>
+  <si>
+    <t>RAHUL</t>
+  </si>
+  <si>
+    <t>RAKESH</t>
+  </si>
+  <si>
+    <t>ASHISH</t>
+  </si>
+  <si>
+    <t>MANISH</t>
+  </si>
+  <si>
+    <t>DEPARTMENT</t>
+  </si>
+  <si>
+    <t>ELECTRICAL</t>
+  </si>
+  <si>
+    <t>FINANCE</t>
+  </si>
+  <si>
+    <t>POST</t>
+  </si>
+  <si>
+    <t>MANAGER</t>
+  </si>
+  <si>
+    <t>SUPERVISOR</t>
+  </si>
+  <si>
+    <t>PION</t>
+  </si>
+  <si>
+    <t>GUARD</t>
+  </si>
+  <si>
+    <t>CASHER</t>
+  </si>
+  <si>
+    <t>ACCOUNTANT</t>
+  </si>
+  <si>
+    <t>BASIC</t>
+  </si>
+  <si>
+    <t>DA 2.5%</t>
+  </si>
+  <si>
+    <t>Q.1:  HOW MANY EMPLOYEE IN COMPUTER, FINANCE, ELECTRICAL DEPARTMENT.</t>
+  </si>
+  <si>
+    <t>Ans: COMPUTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   FINANCE</t>
+  </si>
+  <si>
+    <t>Q.2: HOW MANY BASIC SALARY IN COMPUTER DEPARTMENT ONLY?</t>
+  </si>
+  <si>
+    <t>Ans:</t>
+  </si>
+  <si>
+    <t>Q.3: MANOJ , ASHISH POST &amp; GRADE</t>
+  </si>
+  <si>
+    <t>HRA 3.5%</t>
+  </si>
+  <si>
+    <t>PF 1.5%</t>
+  </si>
+  <si>
+    <t>Ans:  MANOJ POST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">          MANOJ GRADE</t>
+  </si>
+  <si>
+    <t>ASHISH POST</t>
+  </si>
+  <si>
+    <t>ASHISH GRADE</t>
+  </si>
+  <si>
+    <t>Q.4: IF TOTAL SALARY IS GREATER THEN 20000 THEN "A", IF TOTAL SALARY GREATER THEN 10000 THEN "B", OTHERWISE "C".</t>
+  </si>
+  <si>
+    <t>Q.5: HOW MANY EMPLOYEE IS MANAGER &amp; GUARD?</t>
+  </si>
+  <si>
+    <t>Ans: MANAGER:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">         GUARD:</t>
   </si>
 </sst>
 </file>
@@ -1877,4 +1983,435 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E692DE1-37AE-479C-B23C-7A4A1886ABDB}">
+  <dimension ref="A1:I25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="13.81640625" customWidth="1"/>
+    <col min="3" max="3" width="13.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D4" s="1">
+        <v>5000</v>
+      </c>
+      <c r="E4" s="1">
+        <f>(D4*2.5)/100</f>
+        <v>125</v>
+      </c>
+      <c r="F4" s="1">
+        <f>(D4*3.5)/100</f>
+        <v>175</v>
+      </c>
+      <c r="G4" s="1">
+        <f>(D4*1.5)/100</f>
+        <v>75</v>
+      </c>
+      <c r="H4" s="1">
+        <f>SUM(D4:G4)</f>
+        <v>5375</v>
+      </c>
+      <c r="I4" s="1" t="str">
+        <f>IF(H4&gt;20000,"A",IF(H4&gt;10000,"B","C"))</f>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D5" s="1">
+        <v>8000</v>
+      </c>
+      <c r="E5" s="1">
+        <f t="shared" ref="E5:E11" si="0">(D5*2.5)/100</f>
+        <v>200</v>
+      </c>
+      <c r="F5" s="1">
+        <f t="shared" ref="F5:F11" si="1">(D5*3.5)/100</f>
+        <v>280</v>
+      </c>
+      <c r="G5" s="1">
+        <f t="shared" ref="G5:G11" si="2">(D5*1.5)/100</f>
+        <v>120</v>
+      </c>
+      <c r="H5" s="1">
+        <f t="shared" ref="H5:H11" si="3">SUM(D5:G5)</f>
+        <v>8600</v>
+      </c>
+      <c r="I5" s="1" t="str">
+        <f t="shared" ref="I5:I11" si="4">IF(H5&gt;20000,"A",IF(H5&gt;10000,"B","C"))</f>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="D6" s="1">
+        <v>3000</v>
+      </c>
+      <c r="E6" s="1">
+        <f t="shared" si="0"/>
+        <v>75</v>
+      </c>
+      <c r="F6" s="1">
+        <f t="shared" si="1"/>
+        <v>105</v>
+      </c>
+      <c r="G6" s="1">
+        <f t="shared" si="2"/>
+        <v>45</v>
+      </c>
+      <c r="H6" s="1">
+        <f t="shared" si="3"/>
+        <v>3225</v>
+      </c>
+      <c r="I6" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D7" s="1">
+        <v>6000</v>
+      </c>
+      <c r="E7" s="1">
+        <f t="shared" si="0"/>
+        <v>150</v>
+      </c>
+      <c r="F7" s="1">
+        <f t="shared" si="1"/>
+        <v>210</v>
+      </c>
+      <c r="G7" s="1">
+        <f t="shared" si="2"/>
+        <v>90</v>
+      </c>
+      <c r="H7" s="1">
+        <f t="shared" si="3"/>
+        <v>6450</v>
+      </c>
+      <c r="I7" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="D8" s="1">
+        <v>8000</v>
+      </c>
+      <c r="E8" s="1">
+        <f t="shared" si="0"/>
+        <v>200</v>
+      </c>
+      <c r="F8" s="1">
+        <f t="shared" si="1"/>
+        <v>280</v>
+      </c>
+      <c r="G8" s="1">
+        <f t="shared" si="2"/>
+        <v>120</v>
+      </c>
+      <c r="H8" s="1">
+        <f t="shared" si="3"/>
+        <v>8600</v>
+      </c>
+      <c r="I8" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D9" s="1">
+        <v>9000</v>
+      </c>
+      <c r="E9" s="1">
+        <f t="shared" si="0"/>
+        <v>225</v>
+      </c>
+      <c r="F9" s="1">
+        <f t="shared" si="1"/>
+        <v>315</v>
+      </c>
+      <c r="G9" s="1">
+        <f t="shared" si="2"/>
+        <v>135</v>
+      </c>
+      <c r="H9" s="1">
+        <f t="shared" si="3"/>
+        <v>9675</v>
+      </c>
+      <c r="I9" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D10" s="1">
+        <v>10000</v>
+      </c>
+      <c r="E10" s="1">
+        <f t="shared" si="0"/>
+        <v>250</v>
+      </c>
+      <c r="F10" s="1">
+        <f t="shared" si="1"/>
+        <v>350</v>
+      </c>
+      <c r="G10" s="1">
+        <f t="shared" si="2"/>
+        <v>150</v>
+      </c>
+      <c r="H10" s="1">
+        <f t="shared" si="3"/>
+        <v>10750</v>
+      </c>
+      <c r="I10" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D11" s="1">
+        <v>5000</v>
+      </c>
+      <c r="E11" s="1">
+        <f t="shared" si="0"/>
+        <v>125</v>
+      </c>
+      <c r="F11" s="1">
+        <f t="shared" si="1"/>
+        <v>175</v>
+      </c>
+      <c r="G11" s="1">
+        <f t="shared" si="2"/>
+        <v>75</v>
+      </c>
+      <c r="H11" s="1">
+        <f t="shared" si="3"/>
+        <v>5375</v>
+      </c>
+      <c r="I11" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v>C</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>107</v>
+      </c>
+      <c r="C14">
+        <f>COUNTIF(B3:B11,"COMPUTER")</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>108</v>
+      </c>
+      <c r="C15">
+        <f>COUNTIF(B4:B11,"FINANCE")</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>95</v>
+      </c>
+      <c r="C16">
+        <f>COUNTIF(B4:B11,"ELECTRICAL")</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>110</v>
+      </c>
+      <c r="B18">
+        <f>SUMIF(B4:B11,"COMPUTER",D4:D11)</f>
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>114</v>
+      </c>
+      <c r="C20" t="str">
+        <f>VLOOKUP(A6,A3:H11,3,FALSE)</f>
+        <v>PION</v>
+      </c>
+      <c r="E20" t="s">
+        <v>116</v>
+      </c>
+      <c r="G20" t="str">
+        <f>VLOOKUP(A10,A3:H11,3,FALSE)</f>
+        <v>MANAGER</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>115</v>
+      </c>
+      <c r="C21" t="str">
+        <f>VLOOKUP(A6,A3:I11,9,FALSE)</f>
+        <v>C</v>
+      </c>
+      <c r="E21" t="s">
+        <v>117</v>
+      </c>
+      <c r="G21" t="str">
+        <f>VLOOKUP(A10,A3:I11,9,FALSE)</f>
+        <v>B</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>120</v>
+      </c>
+      <c r="C24">
+        <f>COUNTIF(C4:C11,"MANAGER")</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>121</v>
+      </c>
+      <c r="C25">
+        <f>COUNTIF(C4:C11,"GUARD")</f>
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Day-05: Assignment -05 has completed.
Assignment-05 has completed . I used of Formulas-Sum,If,Counta,Countif,Sumif,Vlookup,Lookup to solve assignment-05.
</commit_message>
<xml_diff>
--- a/Excel-Assignments-solution.xlsx
+++ b/Excel-Assignments-solution.xlsx
@@ -5,18 +5,19 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Analytics\ReClasses\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Analytics\ReClasses\1.Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8F9ADB3-8552-4C42-A158-5F08B5A6793C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2699E63-A8B4-4D40-838D-B97448A789A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{7F6CA21F-FA47-42DF-92A2-56BFE6F74A15}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="4" xr2:uid="{7F6CA21F-FA47-42DF-92A2-56BFE6F74A15}"/>
   </bookViews>
   <sheets>
     <sheet name="Assignment-1" sheetId="1" r:id="rId1"/>
     <sheet name="Assignment-2" sheetId="2" r:id="rId2"/>
     <sheet name="Assignment-3" sheetId="3" r:id="rId3"/>
     <sheet name="Assignment-4" sheetId="4" r:id="rId4"/>
+    <sheet name="Assignment-5" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,8 +37,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="152">
   <si>
     <t>Assigment-1</t>
   </si>
@@ -403,6 +426,96 @@
   </si>
   <si>
     <t xml:space="preserve">         GUARD:</t>
+  </si>
+  <si>
+    <t>Use of Formulas-Sum,If, Counta,Countif,Sumif,Vlookup,Lookup</t>
+  </si>
+  <si>
+    <t>SALESMAN</t>
+  </si>
+  <si>
+    <t>RAMESH</t>
+  </si>
+  <si>
+    <t>AJEET</t>
+  </si>
+  <si>
+    <t>ALOK</t>
+  </si>
+  <si>
+    <t>AMRIT</t>
+  </si>
+  <si>
+    <t>SURENDRA</t>
+  </si>
+  <si>
+    <t>SHASHI</t>
+  </si>
+  <si>
+    <t>JAN</t>
+  </si>
+  <si>
+    <t>FEB</t>
+  </si>
+  <si>
+    <t>MAR</t>
+  </si>
+  <si>
+    <t>APR</t>
+  </si>
+  <si>
+    <t>MAY</t>
+  </si>
+  <si>
+    <t>JUNE</t>
+  </si>
+  <si>
+    <t>SALES</t>
+  </si>
+  <si>
+    <t>TARGET</t>
+  </si>
+  <si>
+    <t>RESULT</t>
+  </si>
+  <si>
+    <t>Q.1: How many Salesman? Salesman Ajeet Target and Result?</t>
+  </si>
+  <si>
+    <t>Ajeet Target</t>
+  </si>
+  <si>
+    <t>Ajeet Result</t>
+  </si>
+  <si>
+    <t>Q.2: If Sales Greater Than Target then Target Achived otherwise Not Achived.</t>
+  </si>
+  <si>
+    <t>Q.3: Rahul,Pooja and Ashok Target &amp; result?</t>
+  </si>
+  <si>
+    <t>Rahul</t>
+  </si>
+  <si>
+    <t>Target</t>
+  </si>
+  <si>
+    <t>Result</t>
+  </si>
+  <si>
+    <t>Pooja</t>
+  </si>
+  <si>
+    <t>Ashok</t>
+  </si>
+  <si>
+    <t>Q.4: How many Salesman Achived Target.</t>
+  </si>
+  <si>
+    <t>Q.5: Which Sales Man Jan Sales 2000 &amp; Feb Sales is 2500?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(Try to help me to solve question 5) </t>
   </si>
 </sst>
 </file>
@@ -2414,4 +2527,574 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{831AA902-77ED-4F87-9B85-B06CD7DAEB69}">
+  <dimension ref="A1:J27"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="11.1796875" customWidth="1"/>
+    <col min="3" max="3" width="11.26953125" customWidth="1"/>
+    <col min="9" max="9" width="11.90625" customWidth="1"/>
+    <col min="10" max="10" width="14.90625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B3" t="s">
+        <v>130</v>
+      </c>
+      <c r="C3" t="s">
+        <v>131</v>
+      </c>
+      <c r="D3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E3" t="s">
+        <v>133</v>
+      </c>
+      <c r="F3" t="s">
+        <v>134</v>
+      </c>
+      <c r="G3" t="s">
+        <v>135</v>
+      </c>
+      <c r="H3" t="s">
+        <v>136</v>
+      </c>
+      <c r="I3" t="s">
+        <v>137</v>
+      </c>
+      <c r="J3" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B4">
+        <v>2000</v>
+      </c>
+      <c r="C4">
+        <v>1500</v>
+      </c>
+      <c r="D4">
+        <v>300</v>
+      </c>
+      <c r="E4">
+        <v>1400</v>
+      </c>
+      <c r="F4">
+        <v>1000</v>
+      </c>
+      <c r="G4">
+        <v>1400</v>
+      </c>
+      <c r="H4">
+        <f>SUM(B4:G4)</f>
+        <v>7600</v>
+      </c>
+      <c r="I4">
+        <v>10000</v>
+      </c>
+      <c r="J4" t="str">
+        <f>IF(H4&gt;I4,"Target Achived","Not Achived")</f>
+        <v>Not Achived</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>91</v>
+      </c>
+      <c r="B5">
+        <v>5000</v>
+      </c>
+      <c r="C5">
+        <v>1200</v>
+      </c>
+      <c r="D5">
+        <v>500</v>
+      </c>
+      <c r="E5">
+        <v>1200</v>
+      </c>
+      <c r="F5">
+        <v>1200</v>
+      </c>
+      <c r="G5">
+        <v>2800</v>
+      </c>
+      <c r="H5">
+        <f t="shared" ref="H5:H14" si="0">SUM(B5:G5)</f>
+        <v>11900</v>
+      </c>
+      <c r="I5">
+        <v>12000</v>
+      </c>
+      <c r="J5" t="str">
+        <f t="shared" ref="J5:J14" si="1">IF(H5&gt;I5,"Target Achived","Not Achived")</f>
+        <v>Not Achived</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>90</v>
+      </c>
+      <c r="B6">
+        <v>3000</v>
+      </c>
+      <c r="C6">
+        <v>800</v>
+      </c>
+      <c r="D6">
+        <v>1200</v>
+      </c>
+      <c r="E6">
+        <v>3000</v>
+      </c>
+      <c r="F6">
+        <v>1500</v>
+      </c>
+      <c r="G6">
+        <v>3500</v>
+      </c>
+      <c r="H6">
+        <f t="shared" si="0"/>
+        <v>13000</v>
+      </c>
+      <c r="I6">
+        <v>18000</v>
+      </c>
+      <c r="J6" t="str">
+        <f t="shared" si="1"/>
+        <v>Not Achived</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>1000</v>
+      </c>
+      <c r="C7">
+        <v>900</v>
+      </c>
+      <c r="D7">
+        <v>1800</v>
+      </c>
+      <c r="E7">
+        <v>5000</v>
+      </c>
+      <c r="F7">
+        <v>1400</v>
+      </c>
+      <c r="G7">
+        <v>1200</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="0"/>
+        <v>11300</v>
+      </c>
+      <c r="I7">
+        <v>10000</v>
+      </c>
+      <c r="J7" t="str">
+        <f t="shared" si="1"/>
+        <v>Target Achived</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>500</v>
+      </c>
+      <c r="C8">
+        <v>1000</v>
+      </c>
+      <c r="D8">
+        <v>2300</v>
+      </c>
+      <c r="E8">
+        <v>8000</v>
+      </c>
+      <c r="F8">
+        <v>1700</v>
+      </c>
+      <c r="G8">
+        <v>1400</v>
+      </c>
+      <c r="H8">
+        <f t="shared" si="0"/>
+        <v>14900</v>
+      </c>
+      <c r="I8">
+        <v>12000</v>
+      </c>
+      <c r="J8" t="str">
+        <f t="shared" si="1"/>
+        <v>Target Achived</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9">
+        <v>800</v>
+      </c>
+      <c r="C9">
+        <v>500</v>
+      </c>
+      <c r="D9">
+        <v>2400</v>
+      </c>
+      <c r="E9">
+        <v>1900</v>
+      </c>
+      <c r="F9">
+        <v>1800</v>
+      </c>
+      <c r="G9">
+        <v>1800</v>
+      </c>
+      <c r="H9">
+        <f t="shared" si="0"/>
+        <v>9200</v>
+      </c>
+      <c r="I9">
+        <v>10000</v>
+      </c>
+      <c r="J9" t="str">
+        <f t="shared" si="1"/>
+        <v>Not Achived</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>125</v>
+      </c>
+      <c r="B10">
+        <v>1200</v>
+      </c>
+      <c r="C10">
+        <v>1400</v>
+      </c>
+      <c r="D10">
+        <v>1500</v>
+      </c>
+      <c r="E10">
+        <v>700</v>
+      </c>
+      <c r="F10">
+        <v>2500</v>
+      </c>
+      <c r="G10">
+        <v>7000</v>
+      </c>
+      <c r="H10">
+        <f t="shared" si="0"/>
+        <v>14300</v>
+      </c>
+      <c r="I10">
+        <v>12000</v>
+      </c>
+      <c r="J10" t="str">
+        <f t="shared" si="1"/>
+        <v>Target Achived</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>126</v>
+      </c>
+      <c r="B11">
+        <v>1500</v>
+      </c>
+      <c r="C11">
+        <v>1800</v>
+      </c>
+      <c r="D11">
+        <v>1800</v>
+      </c>
+      <c r="E11">
+        <v>1800</v>
+      </c>
+      <c r="F11">
+        <v>300</v>
+      </c>
+      <c r="G11">
+        <v>1500</v>
+      </c>
+      <c r="H11">
+        <f t="shared" si="0"/>
+        <v>8700</v>
+      </c>
+      <c r="I11">
+        <v>10000</v>
+      </c>
+      <c r="J11" t="str">
+        <f t="shared" si="1"/>
+        <v>Not Achived</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>127</v>
+      </c>
+      <c r="B12">
+        <v>1800</v>
+      </c>
+      <c r="C12">
+        <v>2500</v>
+      </c>
+      <c r="D12">
+        <v>1700</v>
+      </c>
+      <c r="E12">
+        <v>1500</v>
+      </c>
+      <c r="F12">
+        <v>2800</v>
+      </c>
+      <c r="G12">
+        <v>1800</v>
+      </c>
+      <c r="H12">
+        <f t="shared" si="0"/>
+        <v>12100</v>
+      </c>
+      <c r="I12">
+        <v>12000</v>
+      </c>
+      <c r="J12" t="str">
+        <f t="shared" si="1"/>
+        <v>Target Achived</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>128</v>
+      </c>
+      <c r="B13">
+        <v>200</v>
+      </c>
+      <c r="C13">
+        <v>3000</v>
+      </c>
+      <c r="D13">
+        <v>1900</v>
+      </c>
+      <c r="E13">
+        <v>1200</v>
+      </c>
+      <c r="F13">
+        <v>1500</v>
+      </c>
+      <c r="G13">
+        <v>3000</v>
+      </c>
+      <c r="H13">
+        <f t="shared" si="0"/>
+        <v>10800</v>
+      </c>
+      <c r="I13">
+        <v>10000</v>
+      </c>
+      <c r="J13" t="str">
+        <f t="shared" si="1"/>
+        <v>Target Achived</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>129</v>
+      </c>
+      <c r="B14">
+        <v>1600</v>
+      </c>
+      <c r="C14">
+        <v>1200</v>
+      </c>
+      <c r="D14">
+        <v>2000</v>
+      </c>
+      <c r="E14">
+        <v>800</v>
+      </c>
+      <c r="F14">
+        <v>1700</v>
+      </c>
+      <c r="G14">
+        <v>800</v>
+      </c>
+      <c r="H14">
+        <f t="shared" si="0"/>
+        <v>8100</v>
+      </c>
+      <c r="I14">
+        <v>10000</v>
+      </c>
+      <c r="J14" t="str">
+        <f t="shared" si="1"/>
+        <v>Not Achived</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>56</v>
+      </c>
+      <c r="B17">
+        <f>COUNTA(A4:A14)</f>
+        <v>11</v>
+      </c>
+      <c r="D17" t="s">
+        <v>140</v>
+      </c>
+      <c r="F17">
+        <f>VLOOKUP(A10,A3:I14,9,FALSE)</f>
+        <v>12000</v>
+      </c>
+      <c r="H17" t="s">
+        <v>141</v>
+      </c>
+      <c r="J17" t="str">
+        <f>VLOOKUP(A10,A3:J14,10,FALSE)</f>
+        <v>Target Achived</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>56</v>
+      </c>
+      <c r="B20" t="s">
+        <v>144</v>
+      </c>
+      <c r="E20" t="s">
+        <v>147</v>
+      </c>
+      <c r="H20" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B21" t="s">
+        <v>145</v>
+      </c>
+      <c r="C21">
+        <f>VLOOKUP(A6,A3:J14,9,FALSE)</f>
+        <v>18000</v>
+      </c>
+      <c r="E21" t="s">
+        <v>145</v>
+      </c>
+      <c r="F21">
+        <f>VLOOKUP(A7,A3:J14,9,FALSE)</f>
+        <v>10000</v>
+      </c>
+      <c r="H21" t="s">
+        <v>145</v>
+      </c>
+      <c r="I21">
+        <f>VLOOKUP(A9,A3:J14,9,FALSE)</f>
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B22" t="s">
+        <v>146</v>
+      </c>
+      <c r="C22" t="str">
+        <f>VLOOKUP(A6,A3:J14,10,FALSE)</f>
+        <v>Not Achived</v>
+      </c>
+      <c r="E22" t="s">
+        <v>146</v>
+      </c>
+      <c r="F22" t="str">
+        <f>VLOOKUP(A7,A3:J14,10,FALSE)</f>
+        <v>Target Achived</v>
+      </c>
+      <c r="H22" t="s">
+        <v>146</v>
+      </c>
+      <c r="I22" t="str">
+        <f>VLOOKUP(A9,A3:J14,10,FALSE)</f>
+        <v>Not Achived</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>56</v>
+      </c>
+      <c r="B24">
+        <f>COUNTIF(J4:J14,"Target Achived")</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>56</v>
+      </c>
+      <c r="B26" t="e" cm="1">
+        <f t="array" ref="B26">_xlfn.XLOOKUP(1,(B3:B14=2000)*(C4:C14=2500),A4:A14,"Not Found",0,)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="B27" t="s">
+        <v>151</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:J1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Day-12: Completed Assignment -12,13.
Completed Assignment-12,13. I used of Formulas- Counta and Vlookup to solve assignment-12 and create pivot table using data to solve assignment-13.
</commit_message>
<xml_diff>
--- a/Excel-Assignments-solution.xlsx
+++ b/Excel-Assignments-solution.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data Analytics\ReClasses\1.Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0518F03-7A81-4A8C-9BA0-63846ADA8D89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B80FA2CA-0521-4194-B106-847123ECE2B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="6" activeTab="10" xr2:uid="{7F6CA21F-FA47-42DF-92A2-56BFE6F74A15}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="8" activeTab="12" xr2:uid="{7F6CA21F-FA47-42DF-92A2-56BFE6F74A15}"/>
   </bookViews>
   <sheets>
     <sheet name="Assignment-1" sheetId="1" r:id="rId1"/>
@@ -24,8 +24,13 @@
     <sheet name="Assignment-9" sheetId="9" r:id="rId9"/>
     <sheet name="Assignment-10" sheetId="10" r:id="rId10"/>
     <sheet name="Assignment-11" sheetId="11" r:id="rId11"/>
+    <sheet name="Assignment-12" sheetId="12" r:id="rId12"/>
+    <sheet name="Assignment-13" sheetId="13" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <pivotCaches>
+    <pivotCache cacheId="7" r:id="rId14"/>
+  </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -66,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="377">
   <si>
     <t>Assigment-1</t>
   </si>
@@ -1086,16 +1091,128 @@
   </si>
   <si>
     <t>Q.2: What is the price of a Caffe Morcha, Size Grade, Tall, Venti?</t>
+  </si>
+  <si>
+    <t>Use of Formulas- Counta and Vlookup</t>
+  </si>
+  <si>
+    <t>Product Name</t>
+  </si>
+  <si>
+    <t>Apples</t>
+  </si>
+  <si>
+    <t>Grapefruit</t>
+  </si>
+  <si>
+    <t>Lemons</t>
+  </si>
+  <si>
+    <t>Lime</t>
+  </si>
+  <si>
+    <t>Oranges</t>
+  </si>
+  <si>
+    <t>Peaches</t>
+  </si>
+  <si>
+    <t>Pears</t>
+  </si>
+  <si>
+    <t>Pineapples</t>
+  </si>
+  <si>
+    <t>Jan</t>
+  </si>
+  <si>
+    <t>Feb</t>
+  </si>
+  <si>
+    <t>Mar</t>
+  </si>
+  <si>
+    <t>Apr</t>
+  </si>
+  <si>
+    <t>May</t>
+  </si>
+  <si>
+    <t>Jun</t>
+  </si>
+  <si>
+    <t>Jul</t>
+  </si>
+  <si>
+    <t>Aug</t>
+  </si>
+  <si>
+    <t>Total Sales</t>
+  </si>
+  <si>
+    <t>Q.1: How many Fruits?</t>
+  </si>
+  <si>
+    <t>Q.2: Fruits Lemons and Pineapples sales in Mar and Jul?</t>
+  </si>
+  <si>
+    <t>Create Pivot Table Using Date</t>
+  </si>
+  <si>
+    <t>Johnson</t>
+  </si>
+  <si>
+    <t>Jones</t>
+  </si>
+  <si>
+    <t>Brown</t>
+  </si>
+  <si>
+    <t>Sales</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>UK</t>
+  </si>
+  <si>
+    <t>USA</t>
+  </si>
+  <si>
+    <t>Quarter</t>
+  </si>
+  <si>
+    <t>Qtr 3</t>
+  </si>
+  <si>
+    <t>Qtr 4</t>
+  </si>
+  <si>
+    <t>Qtr 2</t>
+  </si>
+  <si>
+    <t>Qtr 1</t>
+  </si>
+  <si>
+    <t>Row Labels</t>
+  </si>
+  <si>
+    <t>Grand Total</t>
+  </si>
+  <si>
+    <t>Sum of Sales</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="#,##0;[Red]#,##0"/>
     <numFmt numFmtId="165" formatCode="[$$-409]#,##0.00_ ;\-[$$-409]#,##0.00\ "/>
-    <numFmt numFmtId="169" formatCode="[$$-409]#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="[$$-409]#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="[$$-409]#,##0"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -1166,7 +1283,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1178,13 +1295,19 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1209,6 +1332,297 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Ravindra Pal" refreshedDate="46222.907558796294" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="14" xr:uid="{BADB688A-F744-41BB-82A1-3AFE39BE7142}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A3:D17" sheet="Assignment-13"/>
+  </cacheSource>
+  <cacheFields count="4">
+    <cacheField name="Last Name" numFmtId="0">
+      <sharedItems count="5">
+        <s v="Smith"/>
+        <s v="Johnson"/>
+        <s v="Williams"/>
+        <s v="Jones"/>
+        <s v="Brown"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Sales" numFmtId="166">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="1390" maxValue="19302"/>
+    </cacheField>
+    <cacheField name="Country" numFmtId="0">
+      <sharedItems count="2">
+        <s v="UK"/>
+        <s v="USA"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="Quarter" numFmtId="0">
+      <sharedItems count="4">
+        <s v="Qtr 3"/>
+        <s v="Qtr 4"/>
+        <s v="Qtr 2"/>
+        <s v="Qtr 1"/>
+      </sharedItems>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="14">
+  <r>
+    <x v="0"/>
+    <n v="16753"/>
+    <x v="0"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <n v="14808"/>
+    <x v="1"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <n v="10644"/>
+    <x v="0"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <n v="1390"/>
+    <x v="1"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <n v="4865"/>
+    <x v="1"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <n v="12438"/>
+    <x v="0"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <n v="9339"/>
+    <x v="0"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <n v="18919"/>
+    <x v="1"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <n v="9213"/>
+    <x v="1"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <n v="7433"/>
+    <x v="0"/>
+    <x v="3"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <n v="3255"/>
+    <x v="1"/>
+    <x v="2"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <n v="14867"/>
+    <x v="1"/>
+    <x v="0"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <n v="19302"/>
+    <x v="0"/>
+    <x v="1"/>
+  </r>
+  <r>
+    <x v="0"/>
+    <n v="9698"/>
+    <x v="1"/>
+    <x v="3"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0A90D84F-CDCA-48AA-988F-0F376045D8C1}" name="PivotTable3" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="I8:J13" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="4">
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" numFmtId="166" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="3"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="3"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Sales" fld="1" baseField="0" baseItem="0" numFmtId="166"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0CFDC58F-EA34-4144-A7E1-7A52D42DE7DB}" name="PivotTable2" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="I3:J6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="4">
+    <pivotField showAll="0"/>
+    <pivotField dataField="1" numFmtId="166" showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="3">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Sales" fld="1" baseField="0" baseItem="0" numFmtId="166"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C304DAE8-5087-4250-8BF5-C8F5F200E3FA}" name="PivotTable1" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="F3:G9" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="4">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="4"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" numFmtId="166" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Sales" fld="1" baseField="0" baseItem="0" numFmtId="166"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1516,22 +1930,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -2479,13 +2893,13 @@
       <c r="A4" t="s">
         <v>323</v>
       </c>
-      <c r="B4" s="13">
+      <c r="B4" s="11">
         <v>2.95</v>
       </c>
-      <c r="C4" s="13">
+      <c r="C4" s="11">
         <v>3.75</v>
       </c>
-      <c r="D4" s="13">
+      <c r="D4" s="11">
         <v>4.1500000000000004</v>
       </c>
     </row>
@@ -2493,13 +2907,13 @@
       <c r="A5" t="s">
         <v>324</v>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="11">
         <v>2.95</v>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="11">
         <v>3.65</v>
       </c>
-      <c r="D5" s="13">
+      <c r="D5" s="11">
         <v>4.1500000000000004</v>
       </c>
     </row>
@@ -2507,13 +2921,13 @@
       <c r="A6" t="s">
         <v>325</v>
       </c>
-      <c r="B6" s="13">
+      <c r="B6" s="11">
         <v>3.75</v>
       </c>
-      <c r="C6" s="13">
+      <c r="C6" s="11">
         <v>3.95</v>
       </c>
-      <c r="D6" s="13">
+      <c r="D6" s="11">
         <v>4.25</v>
       </c>
     </row>
@@ -2521,13 +2935,13 @@
       <c r="A7" t="s">
         <v>326</v>
       </c>
-      <c r="B7" s="13">
+      <c r="B7" s="11">
         <v>3.25</v>
       </c>
-      <c r="C7" s="13">
+      <c r="C7" s="11">
         <v>3.95</v>
       </c>
-      <c r="D7" s="13">
+      <c r="D7" s="11">
         <v>4.4000000000000004</v>
       </c>
     </row>
@@ -2535,13 +2949,13 @@
       <c r="A8" t="s">
         <v>327</v>
       </c>
-      <c r="B8" s="13">
+      <c r="B8" s="11">
         <v>3.45</v>
       </c>
-      <c r="C8" s="13">
+      <c r="C8" s="11">
         <v>4.1500000000000004</v>
       </c>
-      <c r="D8" s="13">
+      <c r="D8" s="11">
         <v>4.55</v>
       </c>
     </row>
@@ -2549,13 +2963,13 @@
       <c r="A9" t="s">
         <v>328</v>
       </c>
-      <c r="B9" s="13">
+      <c r="B9" s="11">
         <v>2</v>
       </c>
-      <c r="C9" s="13">
+      <c r="C9" s="11">
         <v>2.4</v>
       </c>
-      <c r="D9" s="13">
+      <c r="D9" s="11">
         <v>2.75</v>
       </c>
     </row>
@@ -2563,13 +2977,13 @@
       <c r="A10" t="s">
         <v>329</v>
       </c>
-      <c r="B10" s="13">
+      <c r="B10" s="11">
         <v>3.95</v>
       </c>
-      <c r="C10" s="13">
+      <c r="C10" s="11">
         <v>4.75</v>
       </c>
-      <c r="D10" s="13">
+      <c r="D10" s="11">
         <v>5.15</v>
       </c>
     </row>
@@ -2577,13 +2991,13 @@
       <c r="A11" t="s">
         <v>330</v>
       </c>
-      <c r="B11" s="13">
+      <c r="B11" s="11">
         <v>2.25</v>
       </c>
-      <c r="C11" s="13">
+      <c r="C11" s="11">
         <v>2.5</v>
       </c>
-      <c r="D11" s="13">
+      <c r="D11" s="11">
         <v>2.75</v>
       </c>
     </row>
@@ -2591,13 +3005,13 @@
       <c r="A12" t="s">
         <v>331</v>
       </c>
-      <c r="B12" s="13">
+      <c r="B12" s="11">
         <v>1.75</v>
       </c>
-      <c r="C12" s="13">
+      <c r="C12" s="11">
         <v>1.95</v>
       </c>
-      <c r="D12" s="13">
+      <c r="D12" s="11">
         <v>2.0499999999999998</v>
       </c>
     </row>
@@ -2681,6 +3095,702 @@
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4192DD51-20C4-42DA-A4C1-A63C8A956BA8}">
+  <dimension ref="A1:J17"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.90625" customWidth="1"/>
+    <col min="2" max="2" width="12.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>341</v>
+      </c>
+      <c r="B3" t="s">
+        <v>350</v>
+      </c>
+      <c r="C3" t="s">
+        <v>351</v>
+      </c>
+      <c r="D3" t="s">
+        <v>352</v>
+      </c>
+      <c r="E3" t="s">
+        <v>353</v>
+      </c>
+      <c r="F3" t="s">
+        <v>354</v>
+      </c>
+      <c r="G3" t="s">
+        <v>355</v>
+      </c>
+      <c r="H3" t="s">
+        <v>356</v>
+      </c>
+      <c r="I3" t="s">
+        <v>357</v>
+      </c>
+      <c r="J3" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>342</v>
+      </c>
+      <c r="B4" s="12">
+        <v>2773</v>
+      </c>
+      <c r="C4" s="12">
+        <v>17462</v>
+      </c>
+      <c r="D4" s="12">
+        <v>5954</v>
+      </c>
+      <c r="E4" s="12">
+        <v>1348</v>
+      </c>
+      <c r="F4" s="12">
+        <v>28158</v>
+      </c>
+      <c r="G4" s="12">
+        <v>28799</v>
+      </c>
+      <c r="H4" s="12">
+        <v>25415</v>
+      </c>
+      <c r="I4" s="12">
+        <v>17227</v>
+      </c>
+      <c r="J4" s="12">
+        <f>SUM(B4:I4)</f>
+        <v>127136</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>343</v>
+      </c>
+      <c r="B5" s="12">
+        <v>12908</v>
+      </c>
+      <c r="C5" s="12">
+        <v>3083</v>
+      </c>
+      <c r="D5" s="12">
+        <v>24492</v>
+      </c>
+      <c r="E5" s="12">
+        <v>5825</v>
+      </c>
+      <c r="F5" s="12">
+        <v>1080</v>
+      </c>
+      <c r="G5" s="12">
+        <v>2188</v>
+      </c>
+      <c r="H5" s="12">
+        <v>11087</v>
+      </c>
+      <c r="I5" s="12">
+        <v>15544</v>
+      </c>
+      <c r="J5" s="12">
+        <f t="shared" ref="J5:J11" si="0">SUM(B5:I5)</f>
+        <v>76207</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>344</v>
+      </c>
+      <c r="B6" s="12">
+        <v>6554</v>
+      </c>
+      <c r="C6" s="12">
+        <v>14262</v>
+      </c>
+      <c r="D6" s="12">
+        <v>8377</v>
+      </c>
+      <c r="E6" s="12">
+        <v>24982</v>
+      </c>
+      <c r="F6" s="12">
+        <v>12184</v>
+      </c>
+      <c r="G6" s="12">
+        <v>6430</v>
+      </c>
+      <c r="H6" s="12">
+        <v>21159</v>
+      </c>
+      <c r="I6" s="12">
+        <v>18597</v>
+      </c>
+      <c r="J6" s="12">
+        <f t="shared" si="0"/>
+        <v>112545</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>345</v>
+      </c>
+      <c r="B7" s="12">
+        <v>28913</v>
+      </c>
+      <c r="C7" s="12">
+        <v>1437</v>
+      </c>
+      <c r="D7" s="12">
+        <v>20019</v>
+      </c>
+      <c r="E7" s="12">
+        <v>13026</v>
+      </c>
+      <c r="F7" s="12">
+        <v>26952</v>
+      </c>
+      <c r="G7" s="12">
+        <v>27076</v>
+      </c>
+      <c r="H7" s="12">
+        <v>7040</v>
+      </c>
+      <c r="I7" s="12">
+        <v>10884</v>
+      </c>
+      <c r="J7" s="12">
+        <f t="shared" si="0"/>
+        <v>135347</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>346</v>
+      </c>
+      <c r="B8" s="12">
+        <v>4768</v>
+      </c>
+      <c r="C8" s="12">
+        <v>7622</v>
+      </c>
+      <c r="D8" s="12">
+        <v>28918</v>
+      </c>
+      <c r="E8" s="12">
+        <v>27141</v>
+      </c>
+      <c r="F8" s="12">
+        <v>3578</v>
+      </c>
+      <c r="G8" s="12">
+        <v>10092</v>
+      </c>
+      <c r="H8" s="12">
+        <v>15207</v>
+      </c>
+      <c r="I8" s="12">
+        <v>12771</v>
+      </c>
+      <c r="J8" s="12">
+        <f t="shared" si="0"/>
+        <v>110097</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>347</v>
+      </c>
+      <c r="B9" s="12">
+        <v>13390</v>
+      </c>
+      <c r="C9" s="12">
+        <v>3611</v>
+      </c>
+      <c r="D9" s="12">
+        <v>6226</v>
+      </c>
+      <c r="E9" s="12">
+        <v>27567</v>
+      </c>
+      <c r="F9" s="12">
+        <v>29962</v>
+      </c>
+      <c r="G9" s="12">
+        <v>2967</v>
+      </c>
+      <c r="H9" s="12">
+        <v>5740</v>
+      </c>
+      <c r="I9" s="12">
+        <v>2137</v>
+      </c>
+      <c r="J9" s="12">
+        <f t="shared" si="0"/>
+        <v>91600</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>348</v>
+      </c>
+      <c r="B10" s="12">
+        <v>17585</v>
+      </c>
+      <c r="C10" s="12">
+        <v>28508</v>
+      </c>
+      <c r="D10" s="12">
+        <v>9614</v>
+      </c>
+      <c r="E10" s="12">
+        <v>17110</v>
+      </c>
+      <c r="F10" s="12">
+        <v>12143</v>
+      </c>
+      <c r="G10" s="12">
+        <v>7365</v>
+      </c>
+      <c r="H10" s="12">
+        <v>24185</v>
+      </c>
+      <c r="I10" s="12">
+        <v>1643</v>
+      </c>
+      <c r="J10" s="12">
+        <f t="shared" si="0"/>
+        <v>118153</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>349</v>
+      </c>
+      <c r="B11" s="12">
+        <v>22579</v>
+      </c>
+      <c r="C11" s="12">
+        <v>16301</v>
+      </c>
+      <c r="D11" s="12">
+        <v>6469</v>
+      </c>
+      <c r="E11" s="12">
+        <v>22050</v>
+      </c>
+      <c r="F11" s="12">
+        <v>8740</v>
+      </c>
+      <c r="G11" s="12">
+        <v>18806</v>
+      </c>
+      <c r="H11" s="12">
+        <v>3334</v>
+      </c>
+      <c r="I11" s="12">
+        <v>3597</v>
+      </c>
+      <c r="J11" s="12">
+        <f t="shared" si="0"/>
+        <v>101876</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>56</v>
+      </c>
+      <c r="B14">
+        <f>COUNTA(A4:A11)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>56</v>
+      </c>
+      <c r="B16" t="s">
+        <v>344</v>
+      </c>
+      <c r="C16">
+        <f>VLOOKUP(B16,A4:J11,4)</f>
+        <v>8377</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
+      <c r="B17" t="s">
+        <v>349</v>
+      </c>
+      <c r="C17">
+        <f>VLOOKUP(B17,A4:J11,7)</f>
+        <v>18806</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16A985D8-7304-4B4E-9AF0-684041844602}">
+  <dimension ref="A1:J17"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="11.26953125" customWidth="1"/>
+    <col min="2" max="2" width="11.453125" customWidth="1"/>
+    <col min="6" max="6" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.453125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
+        <v>361</v>
+      </c>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="F3" s="16" t="s">
+        <v>374</v>
+      </c>
+      <c r="G3" t="s">
+        <v>376</v>
+      </c>
+      <c r="I3" s="16" t="s">
+        <v>374</v>
+      </c>
+      <c r="J3" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="B4" s="15">
+        <v>16753</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="F4" s="17" t="s">
+        <v>364</v>
+      </c>
+      <c r="G4" s="11">
+        <v>8120</v>
+      </c>
+      <c r="I4" s="17" t="s">
+        <v>367</v>
+      </c>
+      <c r="J4" s="11">
+        <v>75909</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="B5" s="15">
+        <v>14808</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="F5" s="17" t="s">
+        <v>362</v>
+      </c>
+      <c r="G5" s="11">
+        <v>24147</v>
+      </c>
+      <c r="I5" s="17" t="s">
+        <v>368</v>
+      </c>
+      <c r="J5" s="11">
+        <v>77015</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="B6" s="15">
+        <v>10644</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="F6" s="17" t="s">
+        <v>363</v>
+      </c>
+      <c r="G6" s="11">
+        <v>18036</v>
+      </c>
+      <c r="I6" s="17" t="s">
+        <v>375</v>
+      </c>
+      <c r="J6" s="11">
+        <v>152924</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="B7" s="15">
+        <v>1390</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>224</v>
+      </c>
+      <c r="G7" s="11">
+        <v>45370</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="B8" s="15">
+        <v>4865</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="F8" s="17" t="s">
+        <v>233</v>
+      </c>
+      <c r="G8" s="11">
+        <v>57251</v>
+      </c>
+      <c r="I8" s="16" t="s">
+        <v>374</v>
+      </c>
+      <c r="J8" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="B9" s="15">
+        <v>12438</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="F9" s="17" t="s">
+        <v>375</v>
+      </c>
+      <c r="G9" s="11">
+        <v>152924</v>
+      </c>
+      <c r="I9" s="17" t="s">
+        <v>373</v>
+      </c>
+      <c r="J9" s="11">
+        <v>29569</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="B10" s="15">
+        <v>9339</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>372</v>
+      </c>
+      <c r="I10" s="17" t="s">
+        <v>372</v>
+      </c>
+      <c r="J10" s="11">
+        <v>23238</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="B11" s="15">
+        <v>18919</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="I11" s="17" t="s">
+        <v>370</v>
+      </c>
+      <c r="J11" s="11">
+        <v>51929</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="B12" s="15">
+        <v>9213</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>371</v>
+      </c>
+      <c r="I12" s="17" t="s">
+        <v>371</v>
+      </c>
+      <c r="J12" s="11">
+        <v>48188</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="B13" s="15">
+        <v>7433</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>373</v>
+      </c>
+      <c r="I13" s="17" t="s">
+        <v>375</v>
+      </c>
+      <c r="J13" s="11">
+        <v>152924</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A14" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="B14" s="15">
+        <v>3255</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A15" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="B15" s="15">
+        <v>14867</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A16" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="B16" s="15">
+        <v>19302</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="B17" s="15">
+        <v>9698</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>373</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2695,22 +3805,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
@@ -3049,15 +4159,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
@@ -3819,18 +4929,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="13" t="s">
         <v>122</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
@@ -5173,15 +6283,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="13" t="s">
         <v>180</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
@@ -5594,30 +6704,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="13" t="s">
         <v>192</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="14" t="s">
         <v>205</v>
       </c>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12" t="s">
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14" t="s">
         <v>146</v>
       </c>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
@@ -6010,16 +7120,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="13" t="s">
         <v>219</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">

</xml_diff>